<commit_message>
Updated raw data and images after revision
</commit_message>
<xml_diff>
--- a/Figure_8F_raw_data.xlsx
+++ b/Figure_8F_raw_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\eigene Paper\Sabrina MreB EzrA DivIVA morphotypes in infection\Virulence\raw data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\Forschungsdaten\MF\MF4\OpenData_Team\publishing-dev\publications\Supplementary_raw_data_-_cell_chaining_in_attenuated_Listeria_monocytogenes_mutants\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F803609-7023-49AD-B1A0-872B66C370A6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF2AF10-F05D-4A75-95FB-EF72192815CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12705" xr2:uid="{1B5AA81B-1097-44B2-952D-0CD5A92A5708}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{085DEE27-C6A6-4BB7-897E-4CB0ED51D9B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -20,14 +20,34 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="17">
   <si>
-    <t xml:space="preserve">i </t>
+    <t>CFU/ml</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>strain</t>
+  </si>
+  <si>
+    <t>i</t>
   </si>
   <si>
     <t>ii</t>
@@ -45,22 +65,16 @@
     <t>P vs wt</t>
   </si>
   <si>
-    <t>with BH</t>
-  </si>
-  <si>
     <t>P vs divIVA</t>
   </si>
   <si>
-    <t>invasion rates</t>
-  </si>
-  <si>
-    <t>relative invasion rates</t>
-  </si>
-  <si>
-    <t>BH</t>
+    <t xml:space="preserve">0 h p. i. </t>
   </si>
   <si>
     <t>wt</t>
+  </si>
+  <si>
+    <t>6 h p. i.</t>
   </si>
   <si>
     <r>
@@ -125,6 +139,9 @@
       <t>divIVA secA2 T123A</t>
     </r>
   </si>
+  <si>
+    <t>with BH</t>
+  </si>
 </sst>
 </file>
 
@@ -183,6 +200,19 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -200,27 +230,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -265,11 +281,20 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Tabelle1!$C$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0 h p. i. </c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="bg1">
-                <a:lumMod val="75000"/>
-              </a:schemeClr>
+              <a:schemeClr val="bg1"/>
             </a:solidFill>
             <a:ln>
               <a:solidFill>
@@ -285,42 +310,42 @@
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>Tabelle1!$B$14:$E$14</c:f>
+                <c:f>Tabelle1!$E$14:$E$17</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="4"/>
                   <c:pt idx="0">
-                    <c:v>0.17075289358340051</c:v>
+                    <c:v>1204.0348832155985</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>3.1685440315934437E-3</c:v>
+                    <c:v>1215.2777460317457</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>7.3027326468362838E-2</c:v>
+                    <c:v>14288.992266776548</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>3.2882400144355131E-2</c:v>
+                    <c:v>16577.286669818226</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>Tabelle1!$B$14:$E$14</c:f>
+                <c:f>Tabelle1!$E$14:$E$17</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="4"/>
                   <c:pt idx="0">
-                    <c:v>0.17075289358340051</c:v>
+                    <c:v>1204.0348832155985</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>3.1685440315934437E-3</c:v>
+                    <c:v>1215.2777460317457</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>7.3027326468362838E-2</c:v>
+                    <c:v>14288.992266776548</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>3.2882400144355131E-2</c:v>
+                    <c:v>16577.286669818226</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -341,7 +366,7 @@
           </c:errBars>
           <c:cat>
             <c:strRef>
-              <c:f>Tabelle1!$B$9:$E$9</c:f>
+              <c:f>Tabelle1!$B$14:$B$17</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -351,38 +376,173 @@
                   <c:v>ΔdivIVA</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>ΔdivIVA secA2 M95I</c:v>
+                  <c:v>ΔdivIVA secA2 T123A</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>ΔdivIVA secA2 T123A</c:v>
+                  <c:v>ΔdivIVA secA2 M95I</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Tabelle1!$B$13:$E$13</c:f>
+              <c:f>Tabelle1!$C$14:$C$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.99999999758204516</c:v>
+                  <c:v>62390</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.4859697679263965E-2</c:v>
+                  <c:v>56780</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.73201146508258708</c:v>
+                  <c:v>85630</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.54873684393151778</c:v>
+                  <c:v>64086.666666666664</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C7D2-4EFA-9A4A-EA8BD0AC7CF0}"/>
+              <c16:uniqueId val="{00000000-4B49-4D41-9AD8-063BF3ACAF1E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Tabelle1!$D$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 h p. i.</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="bg1">
+                <a:lumMod val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Tabelle1!$F$14:$F$17</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="4"/>
+                  <c:pt idx="0">
+                    <c:v>72556.621567802576</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>7284.5458563546235</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>13688.072666863414</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>7040.5965656327735</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Tabelle1!$F$14:$F$17</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="4"/>
+                  <c:pt idx="0">
+                    <c:v>72556.621567802576</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>7284.5458563546235</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>13688.072666863414</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>7040.5965656327735</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Tabelle1!$B$14:$B$17</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>wt</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>ΔdivIVA</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>ΔdivIVA secA2 T123A</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>ΔdivIVA secA2 M95I</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Tabelle1!$D$14:$D$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>486366.66666666669</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14678.333333333334</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>144733.33333333334</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>111500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-4B49-4D41-9AD8-063BF3ACAF1E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -396,11 +556,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="527037520"/>
-        <c:axId val="527037848"/>
+        <c:axId val="482493488"/>
+        <c:axId val="482492504"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="527037520"/>
+        <c:axId val="482493488"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -440,20 +600,19 @@
             <a:endParaRPr lang="de-DE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="527037848"/>
-        <c:crossesAt val="1.0000000000000002E-3"/>
+        <c:crossAx val="482492504"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="527037848"/>
+        <c:axId val="482492504"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
-          <c:max val="10"/>
-          <c:min val="1.0000000000000002E-3"/>
+          <c:min val="1000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -490,7 +649,7 @@
             <a:endParaRPr lang="de-DE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="527037520"/>
+        <c:crossAx val="482493488"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -502,8 +661,40 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -511,7 +702,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1093,23 +1283,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>942975</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Diagramm 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{88E01020-0DF2-4CEC-B111-8886FF262EC2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D024060F-B29B-4CF7-9D89-D35B068B01F7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1131,9 +1321,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1171,7 +1361,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1277,7 +1467,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1419,304 +1609,442 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADCBD619-11AF-4FEB-900F-B0F78434F13A}">
-  <dimension ref="A1:E18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED256DC4-2EB2-46B6-B058-8FE49691A43E}">
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="I2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C3" s="3">
+        <v>61110</v>
+      </c>
+      <c r="D3" s="3">
+        <v>62560</v>
+      </c>
+      <c r="E3" s="3">
+        <v>63500</v>
+      </c>
+      <c r="F3" s="3">
+        <f>AVERAGE(C3:E3)</f>
+        <v>62390</v>
+      </c>
+      <c r="G3" s="3">
+        <f>STDEV(C3:E3)</f>
+        <v>1204.0348832155985</v>
+      </c>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="4">
+        <v>57980</v>
+      </c>
+      <c r="D4" s="4">
+        <v>56810</v>
+      </c>
+      <c r="E4" s="4">
+        <v>55550</v>
+      </c>
+      <c r="F4" s="4">
+        <f t="shared" ref="F4:F10" si="0">AVERAGE(C4:E4)</f>
+        <v>56780</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" ref="G4:G10" si="1">STDEV(C4:E4)</f>
+        <v>1215.2777460317457</v>
+      </c>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="4">
+        <v>75120</v>
+      </c>
+      <c r="D5" s="4">
+        <v>101900</v>
+      </c>
+      <c r="E5" s="4">
+        <v>79870</v>
+      </c>
+      <c r="F5" s="4">
+        <f t="shared" si="0"/>
+        <v>85630</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="1"/>
+        <v>14288.992266776548</v>
+      </c>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="2">
+        <v>76080</v>
+      </c>
+      <c r="D6" s="2">
+        <v>71010</v>
+      </c>
+      <c r="E6" s="2">
+        <v>45170</v>
+      </c>
+      <c r="F6" s="2">
+        <f t="shared" si="0"/>
+        <v>64086.666666666664</v>
+      </c>
+      <c r="G6" s="2">
+        <f t="shared" si="1"/>
+        <v>16577.286669818226</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="3">
+        <v>529600</v>
+      </c>
+      <c r="D7" s="3">
+        <v>526900</v>
+      </c>
+      <c r="E7" s="3">
+        <v>402600</v>
+      </c>
+      <c r="F7" s="3">
+        <f t="shared" si="0"/>
+        <v>486366.66666666669</v>
+      </c>
+      <c r="G7" s="3">
+        <f t="shared" si="1"/>
+        <v>72556.621567802576</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="C8" s="4">
+        <v>22790</v>
+      </c>
+      <c r="D8" s="4">
+        <v>8695</v>
+      </c>
+      <c r="E8" s="4">
+        <v>12550</v>
+      </c>
+      <c r="F8" s="4">
+        <f t="shared" si="0"/>
+        <v>14678.333333333334</v>
+      </c>
+      <c r="G8" s="4">
+        <f t="shared" si="1"/>
+        <v>7284.5458563546235</v>
+      </c>
+      <c r="H8" s="4">
+        <f>TTEST($C$7:$E$7,C8:E8,2,2)</f>
+        <v>3.6139891896861596E-4</v>
+      </c>
+      <c r="I8" s="4">
+        <f>H8*3</f>
+        <v>1.0841967569058478E-3</v>
+      </c>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="4">
+        <v>148700</v>
+      </c>
+      <c r="D9" s="4">
+        <v>156000</v>
+      </c>
+      <c r="E9" s="4">
+        <v>129500</v>
+      </c>
+      <c r="F9" s="4">
+        <f t="shared" si="0"/>
+        <v>144733.33333333334</v>
+      </c>
+      <c r="G9" s="4">
+        <f t="shared" si="1"/>
+        <v>13688.072666863414</v>
+      </c>
+      <c r="H9" s="4">
+        <f t="shared" ref="H9:H10" si="2">TTEST($C$7:$E$7,C9:E9,2,2)</f>
+        <v>1.315115376896443E-3</v>
+      </c>
+      <c r="I9" s="4">
+        <f>H9*2</f>
+        <v>2.6302307537928861E-3</v>
+      </c>
+      <c r="J9" s="4">
+        <f>TTEST($C$8:$E$8,C9:E9,2,2)</f>
+        <v>1.3054946316666473E-4</v>
+      </c>
+      <c r="K9" s="4">
+        <f>J9*1</f>
+        <v>1.3054946316666473E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="C10" s="2">
+        <v>119100</v>
+      </c>
+      <c r="D10" s="2">
+        <v>110200</v>
+      </c>
+      <c r="E10" s="2">
+        <v>105200</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>111500</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" si="1"/>
+        <v>7040.5965656327735</v>
+      </c>
+      <c r="H10" s="2">
+        <f t="shared" si="2"/>
+        <v>8.7822932065636139E-4</v>
+      </c>
+      <c r="I10" s="2">
+        <f>H10*1</f>
+        <v>8.7822932065636139E-4</v>
+      </c>
+      <c r="J10" s="2">
+        <f>TTEST($C$8:$E$8,C10:E10,2,2)</f>
+        <v>7.8003331548984859E-5</v>
+      </c>
+      <c r="K10" s="2">
+        <f>J10*2</f>
+        <v>1.5600666309796972E-4</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="3">
-        <v>2.085360459973463</v>
-      </c>
-      <c r="C3" s="3">
-        <v>3.7651598676957006E-2</v>
-      </c>
-      <c r="D3" s="3">
-        <v>1.3940190601380216</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0.91685912240184764</v>
-      </c>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4">
-        <v>1.6801007556675063</v>
-      </c>
-      <c r="C4" s="4">
-        <v>4.460511679644049E-2</v>
-      </c>
-      <c r="D4" s="4">
-        <v>1.1437109481119261</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0.94479830148619959</v>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5">
-        <v>1.5002344116268167</v>
-      </c>
-      <c r="C5" s="5">
-        <v>4.8646886208020872E-2</v>
-      </c>
-      <c r="D5" s="5">
-        <v>1.3168195718654434</v>
-      </c>
-      <c r="E5" s="5">
-        <v>1.0278237827095065</v>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="3">
+        <f>F3</f>
+        <v>62390</v>
+      </c>
+      <c r="D14" s="3">
+        <f>F7</f>
+        <v>486366.66666666669</v>
+      </c>
+      <c r="E14" s="3">
+        <f>G3</f>
+        <v>1204.0348832155985</v>
+      </c>
+      <c r="F14" s="3">
+        <f>G7</f>
+        <v>72556.621567802576</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1">
-        <f>AVERAGE(B3:B5)</f>
-        <v>1.7552318757559286</v>
-      </c>
-      <c r="C6" s="1">
-        <f t="shared" ref="C6:E6" si="0">AVERAGE(C3:C5)</f>
-        <v>4.3634533893806123E-2</v>
-      </c>
-      <c r="D6" s="1">
-        <f t="shared" si="0"/>
-        <v>1.2848498600384637</v>
-      </c>
-      <c r="E6" s="1">
-        <f t="shared" si="0"/>
-        <v>0.96316040219918453</v>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="4">
+        <f t="shared" ref="C15:C17" si="3">F4</f>
+        <v>56780</v>
+      </c>
+      <c r="D15" s="4">
+        <f t="shared" ref="D15:D17" si="4">F8</f>
+        <v>14678.333333333334</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" ref="E15:E17" si="5">G4</f>
+        <v>1215.2777460317457</v>
+      </c>
+      <c r="F15" s="4">
+        <f t="shared" ref="F15:F17" si="6">G8</f>
+        <v>7284.5458563546235</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="4">
+        <f t="shared" si="3"/>
+        <v>85630</v>
+      </c>
+      <c r="D16" s="4">
+        <f t="shared" si="4"/>
+        <v>144733.33333333334</v>
+      </c>
+      <c r="E16" s="4">
+        <f t="shared" si="5"/>
+        <v>14288.992266776548</v>
+      </c>
+      <c r="F16" s="4">
+        <f t="shared" si="6"/>
+        <v>13688.072666863414</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="1" t="s">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="3">
-        <f>B3/1.75523188</f>
-        <v>1.1880826024954965</v>
-      </c>
-      <c r="C10" s="3">
-        <f t="shared" ref="C10:E10" si="1">C3/1.75523188</f>
-        <v>2.1451068150013894E-2</v>
-      </c>
-      <c r="D10" s="3">
-        <f t="shared" si="1"/>
-        <v>0.79420791977526162</v>
-      </c>
-      <c r="E10" s="3">
-        <f t="shared" si="1"/>
-        <v>0.52235783365662647</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B11" s="4">
-        <f t="shared" ref="B11:E12" si="2">B4/1.75523188</f>
-        <v>0.95719589805280103</v>
-      </c>
-      <c r="C11" s="4">
-        <f t="shared" si="2"/>
-        <v>2.5412663309442904E-2</v>
-      </c>
-      <c r="D11" s="4">
-        <f t="shared" si="2"/>
-        <v>0.65160105689963088</v>
-      </c>
-      <c r="E11" s="4">
-        <f t="shared" si="2"/>
-        <v>0.53827549069254577</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="5">
-        <f t="shared" si="2"/>
-        <v>0.85472149219783811</v>
-      </c>
-      <c r="C12" s="5">
-        <f t="shared" si="2"/>
-        <v>2.7715361578335092E-2</v>
-      </c>
-      <c r="D12" s="5">
-        <f t="shared" si="2"/>
-        <v>0.75022541857286884</v>
-      </c>
-      <c r="E12" s="5">
-        <f t="shared" si="2"/>
-        <v>0.58557720744538122</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="1">
-        <f>AVERAGE(B10:B12)</f>
-        <v>0.99999999758204516</v>
-      </c>
-      <c r="C13" s="1">
-        <f t="shared" ref="C13:E13" si="3">AVERAGE(C10:C12)</f>
-        <v>2.4859697679263965E-2</v>
-      </c>
-      <c r="D13" s="1">
+      <c r="C17" s="2">
         <f t="shared" si="3"/>
-        <v>0.73201146508258708</v>
-      </c>
-      <c r="E13" s="1">
-        <f t="shared" si="3"/>
-        <v>0.54873684393151778</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="1">
-        <f>STDEV(B10:B12)</f>
-        <v>0.17075289358340051</v>
-      </c>
-      <c r="C14" s="1">
-        <f t="shared" ref="C14:E14" si="4">STDEV(C10:C12)</f>
-        <v>3.1685440315934437E-3</v>
-      </c>
-      <c r="D14" s="1">
+        <v>64086.666666666664</v>
+      </c>
+      <c r="D17" s="2">
         <f t="shared" si="4"/>
-        <v>7.3027326468362838E-2</v>
-      </c>
-      <c r="E14" s="1">
-        <f t="shared" si="4"/>
-        <v>3.2882400144355131E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1">
-        <f>TTEST($B$10:$B$12,C10:C12,2,2)</f>
-        <v>5.8664385924746992E-4</v>
-      </c>
-      <c r="D15" s="1">
-        <f t="shared" ref="D15:E15" si="5">TTEST($B$10:$B$12,D10:D12,2,2)</f>
-        <v>6.6810454214169313E-2</v>
-      </c>
-      <c r="E15" s="1">
+        <v>111500</v>
+      </c>
+      <c r="E17" s="2">
         <f t="shared" si="5"/>
-        <v>1.086531835861012E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2">
-        <f>C15*3</f>
-        <v>1.7599315777424096E-3</v>
-      </c>
-      <c r="D16" s="2">
-        <f>D15*1</f>
-        <v>6.6810454214169313E-2</v>
-      </c>
-      <c r="E16" s="2">
-        <f>E15*2</f>
-        <v>2.1730636717220239E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2">
-        <f>TTEST($C$10:$C$12,D10:D12,2,2)</f>
-        <v>7.4334667894495837E-5</v>
-      </c>
-      <c r="E17" s="2">
-        <f>TTEST($C$10:$C$12,E10:E12,2,2)</f>
-        <v>1.0448283971437137E-5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2">
-        <f>D17*1</f>
-        <v>7.4334667894495837E-5</v>
-      </c>
-      <c r="E18" s="2">
-        <f>E17*2</f>
-        <v>2.0896567942874273E-5</v>
+        <v>16577.286669818226</v>
+      </c>
+      <c r="F17" s="2">
+        <f t="shared" si="6"/>
+        <v>7040.5965656327735</v>
       </c>
     </row>
   </sheetData>

</xml_diff>